<commit_message>
Retrait de l'export CSV
</commit_message>
<xml_diff>
--- a/grossistes_a_importer.xlsx
+++ b/grossistes_a_importer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulesTADEJ\Desktop\geocodage_fff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_0315D663155DD935D102D8F0505ED87656CC5C64" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2D96DC2-6E78-4CAC-A2BB-698E9332929E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1809,6 +1809,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="14" max="14" width="43.5546875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -4621,5 +4624,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>